<commit_message>
Added Naming consistency with subject folder for refrence question bank excel
</commit_message>
<xml_diff>
--- a/Evaluation/question_bank.xlsx
+++ b/Evaluation/question_bank.xlsx
@@ -514,7 +514,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -531,7 +531,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -548,7 +548,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -566,7 +566,7 @@
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -585,7 +585,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -602,7 +602,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -659,7 +659,7 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -681,7 +681,7 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -703,7 +703,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -721,7 +721,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -739,7 +739,7 @@
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -759,7 +759,7 @@
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -778,7 +778,7 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -796,7 +796,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -814,7 +814,7 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -833,7 +833,7 @@
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -852,7 +852,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -869,7 +869,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Computing and Society</t>
+          <t>computer and society</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="22" ht="75" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -909,7 +909,7 @@
     <row r="23" ht="75" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -930,7 +930,7 @@
     <row r="24" ht="75" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -951,7 +951,7 @@
     <row r="25" ht="105" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -974,7 +974,7 @@
     <row r="26" ht="90" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
     <row r="27" ht="105" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1021,7 +1021,7 @@
     <row r="28" ht="120" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1046,7 +1046,7 @@
     <row r="29" ht="105" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1070,7 +1070,7 @@
     <row r="30" ht="135" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1096,7 +1096,7 @@
     <row r="31" ht="120" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1121,7 +1121,7 @@
     <row r="32" ht="60" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1141,7 +1141,7 @@
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1161,7 +1161,7 @@
     <row r="34" ht="45" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1181,7 +1181,7 @@
     <row r="35" ht="60" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1202,7 +1202,7 @@
     <row r="36" ht="45" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1221,7 +1221,7 @@
     <row r="37" ht="60" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="38" ht="60" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1261,7 +1261,7 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1279,7 +1279,7 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1297,7 +1297,7 @@
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>HCI</t>
+          <t>hci</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1315,7 +1315,7 @@
     <row r="42" ht="105" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1334,7 +1334,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1351,7 +1351,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1368,7 +1368,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1385,7 +1385,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1402,7 +1402,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1419,7 +1419,7 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1436,7 +1436,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1453,7 +1453,7 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1470,7 +1470,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -1504,7 +1504,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -1521,7 +1521,7 @@
     <row r="54" ht="120" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -1542,7 +1542,7 @@
     <row r="55" ht="75" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -1563,7 +1563,7 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -1580,7 +1580,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -1597,7 +1597,7 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -1614,7 +1614,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -1631,7 +1631,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -1648,7 +1648,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Computer System Security</t>
+          <t>computer system security</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -1665,7 +1665,7 @@
     <row r="62" ht="45" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -1684,7 +1684,7 @@
     <row r="63" ht="45" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -1703,7 +1703,7 @@
     <row r="64" ht="60" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -1723,7 +1723,7 @@
     <row r="65" ht="45" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -1742,7 +1742,7 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -1760,7 +1760,7 @@
     <row r="67" ht="135" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="68" ht="150" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -1813,7 +1813,7 @@
     <row r="69" ht="120" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -1837,7 +1837,7 @@
     <row r="70" ht="165" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -1864,7 +1864,7 @@
     <row r="71" ht="165" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -1892,7 +1892,7 @@
     <row r="72" ht="75" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -1913,7 +1913,7 @@
     <row r="73" ht="45" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -1932,7 +1932,7 @@
     <row r="74" ht="75" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -1953,7 +1953,7 @@
     <row r="75" ht="60" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -1973,7 +1973,7 @@
     <row r="76" ht="45" customHeight="1">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -1993,7 +1993,7 @@
     <row r="77" ht="75" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -2015,7 +2015,7 @@
     <row r="78" ht="75" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -2037,7 +2037,7 @@
     <row r="79" ht="75" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -2059,7 +2059,7 @@
     <row r="80" ht="75" customHeight="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -2081,7 +2081,7 @@
     <row r="81" ht="90" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Digital Image Processing</t>
+          <t>digital image</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -2103,7 +2103,7 @@
     <row r="82" ht="165" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -2130,7 +2130,7 @@
     <row r="83" ht="180" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -2158,7 +2158,7 @@
     <row r="84" ht="105" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -2181,7 +2181,7 @@
     <row r="85" ht="225" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -2213,7 +2213,7 @@
     <row r="86" ht="240" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -2245,7 +2245,7 @@
     <row r="87" ht="120" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -2269,7 +2269,7 @@
     <row r="88" ht="285" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -2304,7 +2304,7 @@
     <row r="89" ht="90" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -2326,7 +2326,7 @@
     <row r="90" ht="90" customHeight="1">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -2348,7 +2348,7 @@
     <row r="91" ht="270" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -2382,7 +2382,7 @@
     <row r="92" ht="409.5" customHeight="1">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -2426,7 +2426,7 @@
     <row r="93" ht="240" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -2458,7 +2458,7 @@
     <row r="94" ht="105" customHeight="1">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -2481,7 +2481,7 @@
     <row r="95" ht="105" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -2504,7 +2504,7 @@
     <row r="96" ht="105" customHeight="1">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -2527,7 +2527,7 @@
     <row r="97" ht="60" customHeight="1">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -2547,7 +2547,7 @@
     <row r="98" ht="120" customHeight="1">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -2571,7 +2571,7 @@
     <row r="99" ht="90" customHeight="1">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -2593,7 +2593,7 @@
     <row r="100" ht="75" customHeight="1">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -2615,7 +2615,7 @@
     <row r="101" ht="90" customHeight="1">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>Communication Skills</t>
+          <t>communication skills</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -2637,7 +2637,7 @@
     <row r="102" ht="240" customHeight="1">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="103" ht="210" customHeight="1">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -2681,7 +2681,7 @@
     <row r="104" ht="240" customHeight="1">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -2700,7 +2700,7 @@
     <row r="105" ht="240" customHeight="1">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -2722,7 +2722,7 @@
     <row r="106" ht="270" customHeight="1">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -2742,7 +2742,7 @@
     <row r="107" ht="225" customHeight="1">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -2761,7 +2761,7 @@
     <row r="108" ht="270" customHeight="1">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
@@ -2781,7 +2781,7 @@
     <row r="109" ht="285" customHeight="1">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -2804,7 +2804,7 @@
     <row r="110" ht="330" customHeight="1">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -2824,7 +2824,7 @@
     <row r="111" ht="270" customHeight="1">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
@@ -2845,7 +2845,7 @@
     <row r="112" ht="270" customHeight="1">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="113" ht="240" customHeight="1">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
@@ -2886,7 +2886,7 @@
     <row r="114" ht="255" customHeight="1">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
@@ -2905,7 +2905,7 @@
     <row r="115" ht="270" customHeight="1">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
@@ -2926,7 +2926,7 @@
     <row r="116" ht="270" customHeight="1">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
@@ -2946,7 +2946,7 @@
     <row r="117" ht="270" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
@@ -2966,7 +2966,7 @@
     <row r="118" ht="240" customHeight="1">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="119" ht="285" customHeight="1">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -3008,7 +3008,7 @@
     <row r="120" ht="300" customHeight="1">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -3029,7 +3029,7 @@
     <row r="121" ht="345" customHeight="1">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>Theory of Computation</t>
+          <t>theory of computation</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -3050,7 +3050,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -3067,7 +3067,7 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
@@ -3084,7 +3084,7 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
@@ -3101,7 +3101,7 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -3118,7 +3118,7 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -3135,7 +3135,7 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
@@ -3152,7 +3152,7 @@
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
@@ -3169,7 +3169,7 @@
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
@@ -3186,7 +3186,7 @@
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
@@ -3203,7 +3203,7 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
@@ -3220,7 +3220,7 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
@@ -3237,7 +3237,7 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -3254,7 +3254,7 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
@@ -3271,7 +3271,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -3288,7 +3288,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -3305,7 +3305,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -3322,7 +3322,7 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -3339,7 +3339,7 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -3356,7 +3356,7 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
@@ -3373,7 +3373,7 @@
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>Structure of Programming Language</t>
+          <t>structure of programming language</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -3390,7 +3390,7 @@
     <row r="142" ht="285" customHeight="1">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -3415,7 +3415,7 @@
     <row r="143" ht="270" customHeight="1">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
@@ -3435,7 +3435,7 @@
     <row r="144" ht="240" customHeight="1">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
@@ -3456,7 +3456,7 @@
     <row r="145" ht="345" customHeight="1">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
@@ -3480,7 +3480,7 @@
     <row r="146" ht="225" customHeight="1">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
@@ -3502,7 +3502,7 @@
     <row r="147" ht="315" customHeight="1">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
@@ -3524,7 +3524,7 @@
     <row r="148" ht="300" customHeight="1">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
@@ -3549,7 +3549,7 @@
     <row r="149" ht="270" customHeight="1">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
@@ -3571,7 +3571,7 @@
     <row r="150" ht="300" customHeight="1">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
@@ -3591,7 +3591,7 @@
     <row r="151" ht="285" customHeight="1">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
@@ -3615,7 +3615,7 @@
     <row r="152" ht="285" customHeight="1">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
@@ -3639,7 +3639,7 @@
     <row r="153" ht="375" customHeight="1">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
@@ -3661,7 +3661,7 @@
     <row r="154" ht="409.5" customHeight="1">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
@@ -3688,7 +3688,7 @@
     <row r="155" ht="409.5" customHeight="1">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
@@ -3711,7 +3711,7 @@
     <row r="156" ht="409.5" customHeight="1">
       <c r="A156" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
@@ -3739,7 +3739,7 @@
     <row r="157" ht="330" customHeight="1">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
@@ -3761,7 +3761,7 @@
     <row r="158" ht="405" customHeight="1">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
@@ -3784,7 +3784,7 @@
     <row r="159" ht="345" customHeight="1">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
@@ -3811,7 +3811,7 @@
     <row r="160" ht="390" customHeight="1">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
@@ -3838,7 +3838,7 @@
     <row r="161" ht="360" customHeight="1">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>Embedded Systems</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
@@ -3864,7 +3864,7 @@
     <row r="162" ht="195" customHeight="1">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
@@ -3882,7 +3882,7 @@
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
@@ -3899,7 +3899,7 @@
     <row r="164">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
@@ -3916,7 +3916,7 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
@@ -3933,7 +3933,7 @@
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
@@ -3950,7 +3950,7 @@
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
@@ -3967,7 +3967,7 @@
     <row r="168" ht="165" customHeight="1">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
@@ -3984,7 +3984,7 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
@@ -4001,7 +4001,7 @@
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
@@ -4018,7 +4018,7 @@
     <row r="171" ht="240" customHeight="1">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
@@ -4036,7 +4036,7 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -4053,7 +4053,7 @@
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
@@ -4070,7 +4070,7 @@
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
@@ -4087,7 +4087,7 @@
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
@@ -4104,7 +4104,7 @@
     <row r="176" ht="210" customHeight="1">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
@@ -4121,7 +4121,7 @@
     <row r="177" ht="165" customHeight="1">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
@@ -4140,7 +4140,7 @@
     <row r="178" ht="195" customHeight="1">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
@@ -4160,7 +4160,7 @@
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
@@ -4177,7 +4177,7 @@
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
@@ -4194,7 +4194,7 @@
     <row r="181" ht="409.5" customHeight="1">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>Computer Graphics</t>
+          <t>computer graphics</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
@@ -4219,7 +4219,7 @@
     <row r="182">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
@@ -4236,7 +4236,7 @@
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
@@ -4253,7 +4253,7 @@
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
@@ -4270,7 +4270,7 @@
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
@@ -4287,7 +4287,7 @@
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
@@ -4304,7 +4304,7 @@
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
@@ -4321,7 +4321,7 @@
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
@@ -4338,7 +4338,7 @@
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
@@ -4355,7 +4355,7 @@
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
@@ -4372,7 +4372,7 @@
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
@@ -4389,7 +4389,7 @@
     <row r="192">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
@@ -4406,7 +4406,7 @@
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
@@ -4423,7 +4423,7 @@
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B194" s="3" t="inlineStr">
@@ -4440,7 +4440,7 @@
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B195" s="3" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="196">
       <c r="A196" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B196" s="3" t="inlineStr">
@@ -4474,7 +4474,7 @@
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B197" s="3" t="inlineStr">
@@ -4491,7 +4491,7 @@
     <row r="198">
       <c r="A198" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B198" s="3" t="inlineStr">
@@ -4508,7 +4508,7 @@
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B199" s="3" t="inlineStr">
@@ -4525,7 +4525,7 @@
     <row r="200">
       <c r="A200" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B200" s="3" t="inlineStr">
@@ -4542,7 +4542,7 @@
     <row r="201">
       <c r="A201" s="3" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>operating systems</t>
         </is>
       </c>
       <c r="B201" s="3" t="inlineStr">

</xml_diff>